<commit_message>
Finance: Korrektur nach Einwand von Sandy — § 33 UStDV (Kleinbetragsrechnung) uebersehen, F-009 zurueckgezogen
- F-009 war falsch: bei DIN Media stimmt die Anschrift; bei Apple und OpenAI
  ist die Empfaengerangabe nach § 33 UStDV bis 250 EUR brutto gar nicht
  erforderlich. 17 von 18 Belegen liegen darunter.
- Verfahrensdokumentation: Schritt 2b neu — erst Betragsgrenze, dann
  Pflichtangaben, mit den vier Ausnahmen (u.a. Reverse Charge)
- Rechnungsjournal: offen 12,29 EUR statt strittig 14,76 EUR,
  unstrittig abziehbar 29,97 EUR statt 27,50 EUR
- Bewertung Punkt 4.7 unveraendert 85/100

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q9Ufw3gp3JpDKA5YR2JxGM
</commit_message>
<xml_diff>
--- a/docs/kostenuebersicht-finance.xlsx
+++ b/docs/kostenuebersicht-finance.xlsx
@@ -4013,11 +4013,11 @@
       <c r="R24" s="130" t="n"/>
       <c r="S24" s="111" t="inlineStr">
         <is>
-          <t>davon STRITTIG — Abzug erst nach Klaerung (Belege 2026-001, -004, -009, -012) →</t>
+          <t>davon noch OFFEN — aus zwei verschiedenen Gruenden (Belege 2026-001, -009, -012) →</t>
         </is>
       </c>
       <c r="T24" s="111">
-        <f>ROUND(T5+T8+T13+T16,2)</f>
+        <f>ROUND(T5+T13+T16,2)</f>
         <v/>
       </c>
     </row>
@@ -4071,7 +4071,7 @@
       <c r="R26" s="130" t="n"/>
       <c r="S26" s="130" t="inlineStr">
         <is>
-          <t>Warum strittig — unter § 19 war das egal, unter Regelbesteuerung kostet jeder dieser Punkte den Abzug: 2026-001 und 2026-009 (Apple/Claude Pro) laufen auf "Krampasplatz 4b, 14199 Berlin", nicht auf die Betriebsanschrift Wielandstr. 11 — und die geschaeftliche Veranlassung des Abos ist ohnehin als auffaellig vermerkt. 2026-004 (OpenAI) nennt als Empfaenger "Hugo, Wielandstraße 11" — der Kontoinhaber ist geklaert, der NAME auf der Rechnung ist es nicht; § 14 Abs. 4 Nr. 1 UStG verlangt den vollstaendigen Namen des Leistungsempfaengers. 2026-012 (IONOS) betrifft ausweislich der Zeile drei fremde Domains, Sofortangebot-Anteil 0,00 € — insoweit keine betriebliche Veranlassung. Jeweils moegliche Abhilfe: berichtigte Rechnung beim Anbieter anfordern bzw. den betrieblichen Anteil belegen. Gehoert auf den Steuerberater-Termin.</t>
+          <t>KORREKTUR 17.09.2026 (Head of Finance), nach einem berechtigten Einwand von Sandy: Die erste Fassung dieser Zeilen hat 14,76 EUR als strittig gefuehrt und dabei die KLEINBETRAGSREGELUNG uebersehen. Nach § 33 UStDV braucht eine Rechnung bis 250 EUR brutto WEDER Namen NOCH Anschrift des Leistungsempfaengers — nur Lieferant, Datum, Leistung, Bruttobetrag und Steuersatz. Damit ist Beleg 2026-004 (OpenAI, "Hugo", 15,50 EUR brutto) vollstaendig abzugsfaehig, und bei den Apple-Belegen ist die abweichende Anschrift ebenfalls unschaedlich. Fast alle Belege dieses Betriebs liegen unter 250 EUR. ES BLEIBEN ZWEI ECHTE PUNKTE, beide KEINE Formfehler: (1) 2026-001 und 2026-009, Claude Pro ueber Apple, zusammen 7,02 EUR — offen ist die BETRIEBLICHE VERANLASSUNG (geschaeftlich oder privat genutzt), seit 02.09. vermerkt. (2) 2026-012, IONOS, 5,27 EUR — die Rechnung betrifft drei fremde Domains, Sofortangebot-Anteil 0,00 EUR, also insoweit keine betriebliche Veranlassung. Ausnahme von § 33 UStDV, die hier nicht greift: bei Reverse-Charge-Umsaetzen (§ 13b) gilt die Erleichterung NICHT — die Supabase-Belege brauchen weiter volle Angaben.</t>
         </is>
       </c>
     </row>

</xml_diff>